<commit_message>
Add Taj special price alert
</commit_message>
<xml_diff>
--- a/Taj_Price_History.xlsx
+++ b/Taj_Price_History.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H293"/>
+  <dimension ref="A1:H294"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -9821,6 +9821,38 @@
         </is>
       </c>
     </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>2026-09-13 13:07:10</t>
+        </is>
+      </c>
+      <c r="B294" t="n">
+        <v>13131</v>
+      </c>
+      <c r="C294" t="n">
+        <v>14590</v>
+      </c>
+      <c r="D294" t="n">
+        <v>14031</v>
+      </c>
+      <c r="E294" t="n">
+        <v>15590</v>
+      </c>
+      <c r="F294" t="n">
+        <v>13131</v>
+      </c>
+      <c r="G294" t="inlineStr">
+        <is>
+          <t>SUPERIOR ROOM TWIN BED</t>
+        </is>
+      </c>
+      <c r="H294" t="inlineStr">
+        <is>
+          <t>MEMBER</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Taj price history
</commit_message>
<xml_diff>
--- a/Taj_Price_History.xlsx
+++ b/Taj_Price_History.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1221"/>
+  <dimension ref="A1:H1222"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -39517,6 +39517,38 @@
         </is>
       </c>
     </row>
+    <row r="1222">
+      <c r="A1222" t="inlineStr">
+        <is>
+          <t>2026-10-04 13:01:27</t>
+        </is>
+      </c>
+      <c r="B1222" t="n">
+        <v>9036</v>
+      </c>
+      <c r="C1222" t="n">
+        <v>10040</v>
+      </c>
+      <c r="D1222" t="n">
+        <v>9936</v>
+      </c>
+      <c r="E1222" t="n">
+        <v>11040</v>
+      </c>
+      <c r="F1222" t="n">
+        <v>9036</v>
+      </c>
+      <c r="G1222" t="inlineStr">
+        <is>
+          <t>SUPERIOR ROOM TWIN BED</t>
+        </is>
+      </c>
+      <c r="H1222" t="inlineStr">
+        <is>
+          <t>MEMBER</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>